<commit_message>
update Miocene GPTS age model data column names
</commit_message>
<xml_diff>
--- a/data/Miocene_GPTS_reversals_GTS_age_models.xlsx
+++ b/data/Miocene_GPTS_reversals_GTS_age_models.xlsx
@@ -5,18 +5,18 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\uol.le.ac.uk\root\staff\home\t\twwh1\My Documents\GitHub\shiny_stratigraphy\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\twwh1\GitHub\evolving_age_models\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3797E7DE-B4C4-488B-A19D-40A30AFA0301}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C1848D8-29B4-4257-B081-8EF2184FCE50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-2895" windowWidth="29040" windowHeight="15840" xr2:uid="{EABBE038-32C2-2345-AF9A-99F1DF7CF68D}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11620" xr2:uid="{EABBE038-32C2-2345-AF9A-99F1DF7CF68D}"/>
   </bookViews>
   <sheets>
-    <sheet name="Preliminary MioOcean GPTS" sheetId="1" r:id="rId1"/>
+    <sheet name="mio_ocean_gpts" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Preliminary MioOcean GPTS'!$A$1:$N$108</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">mio_ocean_gpts!$A$1:$N$108</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,33 +45,9 @@
     <t>Reversal</t>
   </si>
   <si>
-    <t>CK1995</t>
-  </si>
-  <si>
-    <t>GTS2004</t>
-  </si>
-  <si>
-    <t>GTS2012</t>
-  </si>
-  <si>
-    <t>GTS2016</t>
-  </si>
-  <si>
-    <t>L2016</t>
-  </si>
-  <si>
-    <t>B2018</t>
-  </si>
-  <si>
-    <t>GTS2020</t>
-  </si>
-  <si>
     <t>GTS2020 source</t>
   </si>
   <si>
-    <t>W2020</t>
-  </si>
-  <si>
     <t>W2020 source</t>
   </si>
   <si>
@@ -711,10 +687,34 @@
     <t>C8n.1n (y)</t>
   </si>
   <si>
-    <t>magnetochron_base</t>
-  </si>
-  <si>
     <t>Magnetochron_y_o_W2020</t>
+  </si>
+  <si>
+    <t>Magnetochron_base</t>
+  </si>
+  <si>
+    <t>Model_CK1995</t>
+  </si>
+  <si>
+    <t>Model_GTS2004</t>
+  </si>
+  <si>
+    <t>Model_GTS2012</t>
+  </si>
+  <si>
+    <t>Model_GTS2016</t>
+  </si>
+  <si>
+    <t>Model_L2016</t>
+  </si>
+  <si>
+    <t>Model_B2018</t>
+  </si>
+  <si>
+    <t>Model_GTS2020</t>
+  </si>
+  <si>
+    <t>Model_W2020</t>
   </si>
 </sst>
 </file>
@@ -1140,54 +1140,54 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" s="8" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>224</v>
+        <v>215</v>
       </c>
       <c r="C1" s="8" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>218</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>219</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="J1" s="9" t="s">
+        <v>223</v>
+      </c>
+      <c r="K1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="L1" s="9" t="s">
+        <v>224</v>
+      </c>
+      <c r="M1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="N1" s="10" t="s">
         <v>3</v>
-      </c>
-      <c r="G1" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="H1" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="I1" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="J1" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="K1" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="L1" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="M1" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="N1" s="10" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="C2" s="2" t="str">
         <f t="shared" ref="C2:C61" si="0">A2&amp;"/"&amp;A3</f>
@@ -1214,15 +1214,15 @@
         <v>3.5960000000000001</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="C3" s="2" t="str">
         <f t="shared" si="0"/>
@@ -1249,15 +1249,15 @@
         <v>4.1870000000000003</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="C4" s="2" t="str">
         <f t="shared" si="0"/>
@@ -1284,15 +1284,15 @@
         <v>4.3</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="C5" s="2" t="str">
         <f t="shared" si="0"/>
@@ -1320,15 +1320,15 @@
         <v>4.4930000000000003</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="C6" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1355,15 +1355,15 @@
         <v>4.6310000000000002</v>
       </c>
       <c r="M6" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="C7" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1391,15 +1391,15 @@
         <v>4.7990000000000004</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="C8" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1426,15 +1426,15 @@
         <v>4.8959999999999999</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="C9" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1462,15 +1462,15 @@
         <v>4.9969999999999999</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="C10" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1497,15 +1497,15 @@
         <v>5.2350000000000003</v>
       </c>
       <c r="M10" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="C11" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1529,24 +1529,24 @@
         <v>6.0229999999999997</v>
       </c>
       <c r="K11" s="4" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="L11" s="2">
         <v>6.0232153000000004</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="N11" s="3" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="C12" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1574,18 +1574,18 @@
         <v>6.2715712000000003</v>
       </c>
       <c r="M12" s="3" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="N12" s="3" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="C13" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1613,18 +1613,18 @@
         <v>6.3862686000000002</v>
       </c>
       <c r="M13" s="3" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="N13" s="3" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="C14" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1652,18 +1652,18 @@
         <v>6.7269706999999999</v>
       </c>
       <c r="M14" s="3" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="N14" s="3" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="C15" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1691,18 +1691,18 @@
         <v>7.1039915000000002</v>
       </c>
       <c r="M15" s="3" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="N15" s="3" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="C16" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1730,18 +1730,18 @@
         <v>7.2137112999999999</v>
       </c>
       <c r="M16" s="3" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="N16" s="3" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="C17" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1769,18 +1769,18 @@
         <v>7.2616639000000003</v>
       </c>
       <c r="M17" s="3" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="N17" s="3" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="C18" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1808,18 +1808,18 @@
         <v>7.3046540999999996</v>
       </c>
       <c r="M18" s="3" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="N18" s="3" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="C19" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1847,18 +1847,18 @@
         <v>7.4560636999999996</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="N19" s="3" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="C20" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1886,18 +1886,18 @@
         <v>7.4988922999999996</v>
       </c>
       <c r="M20" s="3" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="N20" s="3" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="C21" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1925,18 +1925,18 @@
         <v>7.5372095000000003</v>
       </c>
       <c r="M21" s="3" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="N21" s="3" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="C22" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1964,18 +1964,18 @@
         <v>7.6514163000000002</v>
       </c>
       <c r="M22" s="3" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="N22" s="3" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="C23" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2003,18 +2003,18 @@
         <v>7.7010807999999997</v>
       </c>
       <c r="M23" s="3" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="N23" s="3" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="C24" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2042,18 +2042,18 @@
         <v>8.1072825999999996</v>
       </c>
       <c r="M24" s="3" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="N24" s="3" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="C25" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2081,18 +2081,18 @@
         <v>8.2357492000000008</v>
       </c>
       <c r="M25" s="3" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="N25" s="3" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="C26" s="1" t="str">
         <f>A26&amp;"/"&amp;A27</f>
@@ -2116,21 +2116,21 @@
         <v>8.3000000000000007</v>
       </c>
       <c r="K26" s="1" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="L26" s="2">
         <v>8.3000000000000007</v>
       </c>
       <c r="M26" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="C27" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2158,15 +2158,15 @@
         <v>8.7710000000000008</v>
       </c>
       <c r="M27" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="C28" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2194,15 +2194,15 @@
         <v>9.1050000000000004</v>
       </c>
       <c r="M28" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="C29" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2230,15 +2230,15 @@
         <v>9.3109999999999999</v>
       </c>
       <c r="M29" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="C30" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2266,15 +2266,15 @@
         <v>9.4260000000000002</v>
       </c>
       <c r="M30" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="C31" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2302,15 +2302,15 @@
         <v>9.6470000000000002</v>
       </c>
       <c r="M31" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="C32" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2338,15 +2338,15 @@
         <v>9.7210000000000001</v>
       </c>
       <c r="M32" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="C33" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2374,15 +2374,15 @@
         <v>9.7859999999999996</v>
       </c>
       <c r="M33" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="C34" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2410,15 +2410,15 @@
         <v>9.9369999999999994</v>
       </c>
       <c r="M34" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="C35" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2446,15 +2446,15 @@
         <v>9.984</v>
       </c>
       <c r="M35" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="C36" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2482,15 +2482,15 @@
         <v>11.055999999999999</v>
       </c>
       <c r="M36" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="C37" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2518,15 +2518,15 @@
         <v>11.146000000000001</v>
       </c>
       <c r="M37" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="C38" s="1" t="str">
         <f>A38&amp;"/"&amp;A39</f>
@@ -2554,15 +2554,15 @@
         <v>11.188000000000001</v>
       </c>
       <c r="M38" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="C39" s="1" t="str">
         <f>A39&amp;"/"&amp;A40</f>
@@ -2590,15 +2590,15 @@
         <v>11.592000000000001</v>
       </c>
       <c r="M39" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="C40" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2626,15 +2626,15 @@
         <v>11.657</v>
       </c>
       <c r="M40" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="C41" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2662,15 +2662,15 @@
         <v>12.048999999999999</v>
       </c>
       <c r="M41" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="C42" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2698,15 +2698,15 @@
         <v>12.173999999999999</v>
       </c>
       <c r="M42" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="C43" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2734,15 +2734,15 @@
         <v>12.272</v>
       </c>
       <c r="M43" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="C44" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2770,15 +2770,15 @@
         <v>12.474</v>
       </c>
       <c r="M44" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="C45" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2806,15 +2806,15 @@
         <v>12.734999999999999</v>
       </c>
       <c r="M45" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="C46" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2842,15 +2842,15 @@
         <v>12.77</v>
       </c>
       <c r="M46" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C47" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2878,15 +2878,15 @@
         <v>12.829000000000001</v>
       </c>
       <c r="M47" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="C48" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2914,15 +2914,15 @@
         <v>12.887</v>
       </c>
       <c r="M48" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="49" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A49" s="2" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="C49" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2950,15 +2950,15 @@
         <v>13.032</v>
       </c>
       <c r="M49" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="C50" s="1" t="str">
         <f t="shared" si="0"/>
@@ -2986,15 +2986,15 @@
         <v>13.183</v>
       </c>
       <c r="M50" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="51" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A51" s="2" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="C51" s="1" t="str">
         <f t="shared" si="0"/>
@@ -3022,15 +3022,15 @@
         <v>13.363</v>
       </c>
       <c r="M51" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="52" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="C52" s="1" t="str">
         <f t="shared" si="0"/>
@@ -3058,15 +3058,15 @@
         <v>13.608000000000001</v>
       </c>
       <c r="M52" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="53" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A53" s="2" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="C53" s="1" t="str">
         <f t="shared" si="0"/>
@@ -3094,15 +3094,15 @@
         <v>13.739000000000001</v>
       </c>
       <c r="M53" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="54" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="C54" s="1" t="str">
         <f t="shared" si="0"/>
@@ -3130,15 +3130,15 @@
         <v>14.07</v>
       </c>
       <c r="M54" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="55" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A55" s="2" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="C55" s="1" t="str">
         <f t="shared" si="0"/>
@@ -3166,15 +3166,15 @@
         <v>14.163</v>
       </c>
       <c r="M55" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="56" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="C56" s="1" t="str">
         <f t="shared" si="0"/>
@@ -3202,15 +3202,15 @@
         <v>14.609</v>
       </c>
       <c r="M56" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="57" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="C57" s="1" t="str">
         <f t="shared" si="0"/>
@@ -3238,15 +3238,15 @@
         <v>14.775</v>
       </c>
       <c r="M57" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="58" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="C58" s="1" t="str">
         <f t="shared" si="0"/>
@@ -3274,15 +3274,15 @@
         <v>14.87</v>
       </c>
       <c r="M58" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="59" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="C59" s="1" t="str">
         <f t="shared" si="0"/>
@@ -3306,21 +3306,21 @@
         <v>15.04</v>
       </c>
       <c r="K59" s="1" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="L59" s="2">
         <v>15.032</v>
       </c>
       <c r="M59" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="60" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="C60" s="1" t="str">
         <f t="shared" si="0"/>
@@ -3348,15 +3348,15 @@
         <v>15.16</v>
       </c>
       <c r="M60" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="61" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A61" s="2" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="C61" s="1" t="str">
         <f t="shared" si="0"/>
@@ -3384,15 +3384,15 @@
         <v>15.974</v>
       </c>
       <c r="M61" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="62" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="C62" s="1" t="str">
         <f t="shared" ref="C62:C101" si="1">A62&amp;"/"&amp;A63</f>
@@ -3420,15 +3420,15 @@
         <v>16.268000000000001</v>
       </c>
       <c r="M62" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="63" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A63" s="2" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="C63" s="1" t="str">
         <f t="shared" si="1"/>
@@ -3456,15 +3456,15 @@
         <v>16.303000000000001</v>
       </c>
       <c r="M63" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="64" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A64" s="2" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="C64" s="1" t="str">
         <f t="shared" si="1"/>
@@ -3492,15 +3492,15 @@
         <v>16.472000000000001</v>
       </c>
       <c r="M64" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A65" s="2" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="C65" s="1" t="str">
         <f t="shared" si="1"/>
@@ -3528,15 +3528,15 @@
         <v>16.542999999999999</v>
       </c>
       <c r="M65" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A66" s="2" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="C66" s="1" t="str">
         <f t="shared" si="1"/>
@@ -3564,15 +3564,15 @@
         <v>16.721</v>
       </c>
       <c r="M66" s="3" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A67" s="2" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="C67" s="1" t="str">
         <f t="shared" si="1"/>
@@ -3600,15 +3600,15 @@
         <v>17.234999999999999</v>
       </c>
       <c r="M67" s="3" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A68" s="2" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="C68" s="1" t="str">
         <f t="shared" si="1"/>
@@ -3636,15 +3636,15 @@
         <v>17.533000000000001</v>
       </c>
       <c r="M68" s="3" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
     </row>
     <row r="69" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A69" s="2" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="C69" s="1" t="str">
         <f t="shared" si="1"/>
@@ -3672,15 +3672,15 @@
         <v>17.716999999999999</v>
       </c>
       <c r="M69" s="3" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A70" s="2" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="C70" s="1" t="str">
         <f t="shared" si="1"/>
@@ -3708,15 +3708,15 @@
         <v>17.739999999999998</v>
       </c>
       <c r="M70" s="3" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A71" s="2" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="C71" s="1" t="str">
         <f t="shared" si="1"/>
@@ -3740,21 +3740,21 @@
         <v>18.007000000000001</v>
       </c>
       <c r="K71" s="1" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="L71" s="2">
         <v>18.056000000000001</v>
       </c>
       <c r="M71" s="3" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A72" s="2" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="C72" s="1" t="str">
         <f t="shared" si="1"/>
@@ -3778,21 +3778,21 @@
         <v>18.497</v>
       </c>
       <c r="K72" s="1" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="L72" s="2">
         <v>18.524000000000001</v>
       </c>
       <c r="M72" s="3" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
     </row>
     <row r="73" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A73" s="2" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="C73" s="1" t="str">
         <f t="shared" si="1"/>
@@ -3820,15 +3820,15 @@
         <v>18.748000000000001</v>
       </c>
       <c r="M73" s="3" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
     </row>
     <row r="74" spans="1:14" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A74" s="6" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="C74" s="1" t="str">
         <f t="shared" si="1"/>
@@ -3856,18 +3856,18 @@
         <v>19.726512</v>
       </c>
       <c r="M74" s="7" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="N74" s="7" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="75" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A75" s="2" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="C75" s="1" t="str">
         <f t="shared" si="1"/>
@@ -3895,18 +3895,18 @@
         <v>20.100332999999999</v>
       </c>
       <c r="M75" s="3" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="N75" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="76" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A76" s="2" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="C76" s="1" t="str">
         <f t="shared" si="1"/>
@@ -3930,24 +3930,24 @@
         <v>20.181999999999999</v>
       </c>
       <c r="K76" s="1" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="L76" s="2">
         <v>20.236488999999999</v>
       </c>
       <c r="M76" s="3" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="N76" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="77" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A77" s="2" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="C77" s="1" t="str">
         <f t="shared" si="1"/>
@@ -3975,18 +3975,18 @@
         <v>20.406721999999998</v>
       </c>
       <c r="M77" s="3" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="N77" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="78" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A78" s="2" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="C78" s="1" t="str">
         <f t="shared" si="1"/>
@@ -4010,24 +4010,24 @@
         <v>20.765000000000001</v>
       </c>
       <c r="K78" s="1" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="L78" s="2">
         <v>20.672937999999998</v>
       </c>
       <c r="M78" s="3" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="N78" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="79" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A79" s="2" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="C79" s="1" t="str">
         <f t="shared" si="1"/>
@@ -4051,24 +4051,24 @@
         <v>21.13</v>
       </c>
       <c r="K79" s="1" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="L79" s="2">
         <v>21.058230999999999</v>
       </c>
       <c r="M79" s="3" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="N79" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="80" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A80" s="2" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="C80" s="1" t="str">
         <f t="shared" si="1"/>
@@ -4096,18 +4096,18 @@
         <v>21.202072000000001</v>
       </c>
       <c r="M80" s="3" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="N80" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="81" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A81" s="2" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="C81" s="1" t="str">
         <f t="shared" si="1"/>
@@ -4135,18 +4135,18 @@
         <v>21.487524000000001</v>
       </c>
       <c r="M81" s="3" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="N81" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="82" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A82" s="2" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="C82" s="1" t="str">
         <f t="shared" si="1"/>
@@ -4174,18 +4174,18 @@
         <v>21.544360000000001</v>
       </c>
       <c r="M82" s="3" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="N82" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="83" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A83" s="2" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="C83" s="1" t="str">
         <f t="shared" si="1"/>
@@ -4209,24 +4209,24 @@
         <v>21.690999999999999</v>
       </c>
       <c r="K83" s="1" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="L83" s="2">
         <v>21.687864000000001</v>
       </c>
       <c r="M83" s="3" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="N83" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="84" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A84" s="2" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="C84" s="1" t="str">
         <f t="shared" si="1"/>
@@ -4250,24 +4250,24 @@
         <v>21.722000000000001</v>
       </c>
       <c r="K84" s="1" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="L84" s="2">
         <v>21.73272</v>
       </c>
       <c r="M84" s="3" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="N84" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="85" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A85" s="2" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="C85" s="1" t="str">
         <f t="shared" si="1"/>
@@ -4295,18 +4295,18 @@
         <v>21.785632</v>
       </c>
       <c r="M85" s="3" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="N85" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="86" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A86" s="2" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="C86" s="1" t="str">
         <f t="shared" si="1"/>
@@ -4332,24 +4332,24 @@
         <v>21.984999999999999</v>
       </c>
       <c r="K86" s="1" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="L86" s="2">
         <v>21.99099</v>
       </c>
       <c r="M86" s="3" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="N86" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="87" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A87" s="2" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="C87" s="1" t="str">
         <f t="shared" si="1"/>
@@ -4379,18 +4379,18 @@
         <v>22.050087000000001</v>
       </c>
       <c r="M87" s="3" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="N87" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="88" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A88" s="2" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="C88" s="1" t="str">
         <f t="shared" si="1"/>
@@ -4422,18 +4422,18 @@
         <v>22.312954000000001</v>
       </c>
       <c r="M88" s="3" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="N88" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="89" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A89" s="2" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="C89" s="1" t="str">
         <f t="shared" si="1"/>
@@ -4465,18 +4465,18 @@
         <v>22.626469</v>
       </c>
       <c r="M89" s="3" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="N89" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="90" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A90" s="2" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="C90" s="1" t="str">
         <f t="shared" si="1"/>
@@ -4508,18 +4508,18 @@
         <v>22.794326000000002</v>
       </c>
       <c r="M90" s="3" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="N90" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="91" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A91" s="2" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="C91" s="1" t="str">
         <f t="shared" si="1"/>
@@ -4551,18 +4551,18 @@
         <v>22.957353000000001</v>
       </c>
       <c r="M91" s="3" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="N91" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="92" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A92" s="2" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="C92" s="1" t="str">
         <f t="shared" si="1"/>
@@ -4592,18 +4592,18 @@
         <v>23.039287999999999</v>
       </c>
       <c r="M92" s="3" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="N92" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="93" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A93" s="2" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="C93" s="1" t="str">
         <f t="shared" si="1"/>
@@ -4633,18 +4633,18 @@
         <v>23.214879</v>
       </c>
       <c r="M93" s="3" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="N93" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="94" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A94" s="2" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C94" s="1" t="str">
         <f t="shared" si="1"/>
@@ -4674,18 +4674,18 @@
         <v>23.322583999999999</v>
       </c>
       <c r="M94" s="3" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="N94" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="95" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A95" s="2" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="C95" s="1" t="str">
         <f t="shared" si="1"/>
@@ -4713,18 +4713,18 @@
         <v>24.032212000000001</v>
       </c>
       <c r="M95" s="3" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="N95" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="96" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A96" s="2" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
       <c r="C96" s="1" t="str">
         <f t="shared" si="1"/>
@@ -4752,18 +4752,18 @@
         <v>24.057039</v>
       </c>
       <c r="M96" s="3" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="N96" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="97" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A97" s="2" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="C97" s="1" t="str">
         <f t="shared" si="1"/>
@@ -4791,18 +4791,18 @@
         <v>24.115289000000001</v>
       </c>
       <c r="M97" s="3" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="N97" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="98" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A98" s="2" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="C98" s="1" t="str">
         <f t="shared" si="1"/>
@@ -4828,18 +4828,18 @@
         <v>24.462091999999998</v>
       </c>
       <c r="M98" s="3" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="N98" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="99" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A99" s="2" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="C99" s="1" t="str">
         <f t="shared" si="1"/>
@@ -4865,18 +4865,18 @@
         <v>24.768415999999998</v>
       </c>
       <c r="M99" s="3" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="N99" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="100" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A100" s="2" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="C100" s="1" t="str">
         <f t="shared" si="1"/>
@@ -4902,18 +4902,18 @@
         <v>24.894566000000001</v>
       </c>
       <c r="M100" s="3" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="N100" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="101" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A101" s="2" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>222</v>
+        <v>214</v>
       </c>
       <c r="C101" s="1" t="str">
         <f t="shared" si="1"/>
@@ -4935,16 +4935,16 @@
         <v>25.099</v>
       </c>
       <c r="K101" s="1" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="L101" s="2">
         <v>25.049133999999999</v>
       </c>
       <c r="M101" s="3" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="N101" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
simplified the Miocene gpts data file
</commit_message>
<xml_diff>
--- a/data/Miocene_GPTS_reversals_GTS_age_models.xlsx
+++ b/data/Miocene_GPTS_reversals_GTS_age_models.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\twwh1\GitHub\evolving_age_models\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6A5DC1F-BD75-46DD-8D1C-407B1EE4840F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44E234D7-140B-4C58-9209-0EAE6EEDAF41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11620" xr2:uid="{EABBE038-32C2-2345-AF9A-99F1DF7CF68D}"/>
   </bookViews>
@@ -3846,7 +3846,7 @@
         <v>139</v>
       </c>
       <c r="B67" s="1" t="str">
-        <f t="shared" ref="B67:B101" si="3">A68</f>
+        <f t="shared" ref="B67:B100" si="3">A68</f>
         <v>C5Dn</v>
       </c>
       <c r="C67" s="2" t="s">

</xml_diff>